<commit_message>
feat: Switch from fuzzy matching and data normalization of input file to enforced frictionless schema
</commit_message>
<xml_diff>
--- a/input/rodent_dataset.xlsx
+++ b/input/rodent_dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kassyr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiat\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E213A50D-0CC0-4015-9BF3-34C3FE443494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC7CC205-F3B0-49C7-83F7-80ABC380532F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-220" yWindow="580" windowWidth="18310" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="98">
   <si>
     <t>School Type</t>
   </si>
@@ -296,6 +296,24 @@
   </si>
   <si>
     <t>Ratty</t>
+  </si>
+  <si>
+    <t>1009876548</t>
+  </si>
+  <si>
+    <t>Birth Year</t>
+  </si>
+  <si>
+    <t>2013</t>
+  </si>
+  <si>
+    <t>2012</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>2009</t>
   </si>
 </sst>
 </file>
@@ -354,12 +372,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,17 +684,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.6328125" customWidth="1"/>
     <col min="2" max="2" width="31.26953125" customWidth="1"/>
     <col min="3" max="3" width="22.90625" customWidth="1"/>
-    <col min="7" max="7" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.81640625" customWidth="1"/>
+    <col min="8" max="8" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -694,43 +714,46 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -749,41 +772,44 @@
       <c r="F2">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H2" t="s">
         <v>39</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>44</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>51</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>56</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>57</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>90</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>66</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>70</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>75</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>80</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -802,41 +828,44 @@
       <c r="F3">
         <v>11</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H3" t="s">
         <v>40</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>45</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>52</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>56</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>58</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>62</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>67</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>71</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>76</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>81</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -855,44 +884,47 @@
       <c r="F4">
         <v>13</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" t="s">
         <v>41</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>46</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>49</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>53</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>56</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>59</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>63</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>68</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>72</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>77</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>82</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -911,41 +943,44 @@
       <c r="F5">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H5" t="s">
         <v>42</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>47</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>54</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>56</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>60</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>64</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>67</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>73</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>78</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>83</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -964,52 +999,55 @@
       <c r="F6">
         <v>11</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H6" t="s">
         <v>43</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>48</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>50</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>55</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>56</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>61</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>65</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>69</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>74</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>79</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>84</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>18</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="C7">
-        <v>1009876548</v>
+      <c r="C7" s="3" t="s">
+        <v>92</v>
       </c>
       <c r="D7" t="s">
         <v>91</v>
@@ -1020,34 +1058,37 @@
       <c r="F7">
         <v>17</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H7" s="2">
         <v>39872</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>55</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>56</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>61</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>65</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>69</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
         <v>74</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>79</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>84</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>